<commit_message>
Tokyo guide: N'EX timetable (21 from Shinjuku 11:08 on 10/5, airport departures tonight), 10/2 alert, stale wording
- 10/5: N'EX 21 Shinjuku 11:08 -> Airport Terminal 2 12:27, walk or shuttle to T3 by 12:45;
  alternatives 19 (10:38) and 23 (11:38). Leave the lodging 10:20.
- 10/1 arrival: N'EX departures from the airport this evening, reserve both seats at once.
- Alert refreshed for the evening of 10/1 (typhoon passed; check 10/2 weather and JR status).
- Calendars rebuild days 1 and 5 from the page too (same UIDs, 36 events).
- Workbook, README and N'EX show card updated; SW cache bumped.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AoPkjGThxHgQ4GKNLnhfKD
</commit_message>
<xml_diff>
--- a/tokyo/tokyo-family-final.xlsx
+++ b/tokyo/tokyo-family-final.xlsx
@@ -837,8 +837,9 @@
       <c r="B12" s="5" t="inlineStr">
         <is>
           <t>월요일 · 귀국
-숙소 아침 → 체크아웃
-신주쿠역에서 공항 이동</t>
+09:30 짐 정리·체크아웃 준비
+10:20 숙소 출발(택시) → 신주쿠역
+11:08 N'EX 21호 → 공항제2빌딩 12:27</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -862,10 +863,10 @@
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>11시대 NEX 후보: 실제 열차 확인
-나리타 T3 13:00~13:20 도착 목표
-기존 가이드 16:20 출발 기준
-항공권·터미널은 예약 내역 재확인</t>
+          <t>N'EX 21호(신주쿠 11:08 → 공항제2빌딩 12:27, 평일 시각)
+대안: 11:38 발 23호(12:54) · 10:38 발 19호(11:53)
+제3터미널은 역에서 걸어서 약 15분, 12:45경 도착
+ZE610 16:20 · 10/5는 한국 대체공휴일이라 붐빔</t>
         </is>
       </c>
     </row>
@@ -1678,22 +1679,22 @@
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>출발 전</t>
+          <t>10/1 교환 때</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>편명·터미널·NEX 지정석</t>
+          <t>10/5 N'EX 21호(신주쿠 11:08) 3명 지정석</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>기존 가이드 기준, 재확인 필요</t>
+          <t>바우처 교환 시 지정</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>NEX 11시대는 계획용 구간이지 발권 완료 열차가 아님.</t>
+          <t>지정석 표의 시각이 우선. 21호가 안 되면 23호(11:38) 또는 19호(10:38).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tokyo guide: 10/1 dinner is yakiniku within the family budget (Ushigoro or Aging Beef)
- Day 1 20:15: Yakiniku Ushigoro Shinjuku-sanchome (Tabelog 3.67, Yakiniku
  Hyakumeiten 2025, L.O. 22:30) or Aging Beef Tokyo Shinjuku-sanchome
  (aged wagyu, about 6,200 yen per person, L.O. 22:00), both near the lodging;
  budget 100,000-150,000 KRW for three (about 11,400-17,400 yen). Hayashida
  ramen stays as the quick fallback. Call and map buttons for both.
- Overview, README, workbook (itinerary D8/F8, budget row 19 with cached
  totals) and both calendars (10/1 dinner at SEQUENCE 3) follow.
- Food budget 91,200-136,500 yen, with Air Cabin 96,600-141,900 yen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AoPkjGThxHgQ4GKNLnhfKD
</commit_message>
<xml_diff>
--- a/tokyo/tokyo-family-final.xlsx
+++ b/tokyo/tokyo-family-final.xlsx
@@ -681,8 +681,9 @@
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>20:15 이후 목표
-하야시다 신주쿠 본점
-입국·체크인 후 결정</t>
+고기 저녁(신주쿠산초메)
+① 야키니쿠 우시고로 (L.O. 22:30, 03-3358-4129)
+② 에이징 비프 (L.O. 22:00, 03-6273-2985)</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -693,9 +694,9 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>라멘 대기 20분 이상 → 교자노 후쿠호
-너무 늦으면 편의점·포장 식사
-진로쿠는 저녁 영업 상충으로 보류</t>
+          <t>3명 예산 10~15만 원(약 11,400~17,400엔)
+코스는 상한을 넘으니 단품 위주
+늦거나 피곤하면 하야시다 라멘</t>
         </is>
       </c>
     </row>
@@ -966,24 +967,22 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>라멘 하야시다 신주쿠 본점</t>
-        </is>
-      </c>
-      <c r="C19" s="47">
-        <f>'맛집 상세'!E7</f>
-        <v>1500</v>
-      </c>
-      <c r="D19" s="47">
-        <f>'맛집 상세'!F7</f>
-        <v>2000</v>
+          <t>고기 저녁 (우시고로 또는 에이징 비프, 3명 10~15만 원)</t>
+        </is>
+      </c>
+      <c r="C19" s="47" t="n">
+        <v>3800</v>
+      </c>
+      <c r="D19" s="47" t="n">
+        <v>5800</v>
       </c>
       <c r="E19" s="47">
         <f>C19*$B$17</f>
-        <v>4500</v>
+        <v>11400</v>
       </c>
       <c r="F19" s="47">
         <f>D19*$B$17</f>
-        <v>6000</v>
+        <v>17400</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
@@ -1323,19 +1322,19 @@
       </c>
       <c r="C32" s="48">
         <f>SUM(C19:C31)</f>
-        <v>28100</v>
+        <v>30400</v>
       </c>
       <c r="D32" s="48">
         <f>SUM(D19:D31)</f>
-        <v>41700</v>
+        <v>45500</v>
       </c>
       <c r="E32" s="48">
         <f>SUM(E19:E31)</f>
-        <v>84300</v>
+        <v>91200</v>
       </c>
       <c r="F32" s="48">
         <f>SUM(F19:F31)</f>
-        <v>125100</v>
+        <v>136500</v>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
@@ -1437,19 +1436,19 @@
       </c>
       <c r="C37" s="48">
         <f>C32+C36</f>
-        <v>29900</v>
+        <v>32200</v>
       </c>
       <c r="D37" s="48">
         <f>D32+D36</f>
-        <v>43500</v>
+        <v>47300</v>
       </c>
       <c r="E37" s="48">
         <f>E32+E36</f>
-        <v>89700</v>
+        <v>96600</v>
       </c>
       <c r="F37" s="48">
         <f>F32+F36</f>
-        <v>130500</v>
+        <v>141900</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1">

</xml_diff>

<commit_message>
Tokyo guide: price the 10/1 dinner from listed menu prices; workbook detail row and map point follow
- Day 1 dinner: family target 100,000-150,000 KRW stays, plus what it really
  costs. An in-budget Ushigoro order from menu prices (tongue 1,600 x2, harami
  2,200 x2, uchimomo 1,800 x2, kimchi 880 = about 12,100 yen, about 15,000 with
  rice and drinks). Course and Aging Beef totals are stated as slightly over.
- Budget row: 5,000-7,000 yen per person (15,000-21,000 for three); food
  94,800-140,100 yen, with Air Cabin 100,200-145,500 yen.
- Workbook detail row 7 now holds Ushigoro (and Aging Beef as the alternative,
  Hayashida as fallback); budget row 19 references it again.
- The stop's map point moves to Ushigoro (HULIC &New SHINJUKU).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AoPkjGThxHgQ4GKNLnhfKD
</commit_message>
<xml_diff>
--- a/tokyo/tokyo-family-final.xlsx
+++ b/tokyo/tokyo-family-final.xlsx
@@ -694,8 +694,8 @@
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>3명 예산 10~15만 원(약 11,400~17,400엔)
-코스는 상한을 넘으니 단품 위주
+          <t>가족 목표 3명 10~15만 원(약 11,400~17,400엔)
+단품 약 15,000엔 · 코스+음료 약 21,000엔
 늦거나 피곤하면 하야시다 라멘</t>
         </is>
       </c>
@@ -967,22 +967,24 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>고기 저녁 (우시고로 또는 에이징 비프, 3명 10~15만 원)</t>
-        </is>
-      </c>
-      <c r="C19" s="47" t="n">
-        <v>3800</v>
-      </c>
-      <c r="D19" s="47" t="n">
-        <v>5800</v>
+          <t>고기 저녁 (우시고로 또는 에이징 비프)</t>
+        </is>
+      </c>
+      <c r="C19" s="47">
+        <f>'맛집 상세'!E7</f>
+        <v>5000</v>
+      </c>
+      <c r="D19" s="47">
+        <f>'맛집 상세'!F7</f>
+        <v>7000</v>
       </c>
       <c r="E19" s="47">
         <f>C19*$B$17</f>
-        <v>11400</v>
+        <v>15000</v>
       </c>
       <c r="F19" s="47">
         <f>D19*$B$17</f>
-        <v>17400</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
@@ -1322,19 +1324,19 @@
       </c>
       <c r="C32" s="48">
         <f>SUM(C19:C31)</f>
-        <v>30400</v>
+        <v>31600</v>
       </c>
       <c r="D32" s="48">
         <f>SUM(D19:D31)</f>
-        <v>45500</v>
+        <v>46700</v>
       </c>
       <c r="E32" s="48">
         <f>SUM(E19:E31)</f>
-        <v>91200</v>
+        <v>94800</v>
       </c>
       <c r="F32" s="48">
         <f>SUM(F19:F31)</f>
-        <v>136500</v>
+        <v>140100</v>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
@@ -1436,19 +1438,19 @@
       </c>
       <c r="C37" s="48">
         <f>C32+C36</f>
-        <v>32200</v>
+        <v>33400</v>
       </c>
       <c r="D37" s="48">
         <f>D32+D36</f>
-        <v>47300</v>
+        <v>48500</v>
       </c>
       <c r="E37" s="48">
         <f>E32+E36</f>
-        <v>96600</v>
+        <v>100200</v>
       </c>
       <c r="F37" s="48">
         <f>F32+F36</f>
-        <v>141900</v>
+        <v>145500</v>
       </c>
     </row>
     <row r="38" ht="44" customHeight="1">
@@ -1998,39 +2000,41 @@
       </c>
       <c r="C7" s="29" t="inlineStr">
         <is>
-          <t>라멘 하야시다 신주쿠 본점
-らぁ麺 はやし田 新宿本店
-新宿3-31-5 ペガサス館102
-TEL 03-6380-0047</t>
+          <t>야키니쿠 우시고로 신주쿠산초메점
+焼肉うしごろ 新宿三丁目店
+新宿3-17-10 HULIC &amp;New SHINJUKU 12F
+TEL 03-3358-4129
+(대안) 에이징 비프 TOKYO 신주쿠산초메점
+新宿3-5-4 6F · TEL 03-6273-2985</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>간장 라멘
-오리와 닭을 쓰는 육수가 특징. 도착일에 무거운 코스 대신 한 그릇으로 마무리.</t>
+          <t>흑우 혀(구로탄)·하라미 · 타베로그 3.67, 야키니쿠 백명점 2025
+단품 예시(3명): 혀 1,600×2 + 하라미 2,200×2 + 우치모모 1,800×2 + 김치 모둠 880 = 약 12,100엔, 밥·음료 포함 약 15,000엔</t>
         </is>
       </c>
       <c r="E7" s="49" t="n">
-        <v>1500</v>
+        <v>5000</v>
       </c>
       <c r="F7" s="49" t="n">
-        <v>2000</v>
+        <v>7000</v>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>매일 11:00~23:00
-20:15 이후 도착 상황에 맞춰 방문. 예약 식사로 묶지 않음.</t>
+          <t>우시고로 17:00~23:30 (L.O. 22:30)
+에이징 비프 17:00~23:00 (L.O. 22:00)
+예약 완료 아님 · N’EX 안에서 전화로 확인</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>예상 대기가 20분을 넘으면 교자노 후쿠호로 전환. 입국·수하물 지연 시 맛집보다 체크인과 휴식 우선.</t>
+          <t>가족 목표 3명 10~15만 원(약 11,400~17,400엔). 코스(1인 6,100엔~, 3명 18,300엔)와 에이징 비프(1인 평균 약 6,200엔)는 상한을 조금 넘음. 메뉴판 가격에 세금·서비스료가 따로 붙을 수 있음. 늦거나 피곤하면 하야시다 라멘(1인 1,500~2,000엔, 新宿3-31-5).</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>원본 #136 / 143행
-영업시간·육수: 운영사 공식</t>
+          <t>공식 매장 페이지 · 타베로그 · 一休 코스 · 메뉴 가격 (10/1 확인)</t>
         </is>
       </c>
       <c r="J7" s="31" t="inlineStr">
@@ -2625,7 +2629,7 @@
       <c r="D17" s="5" t="inlineStr">
         <is>
           <t>군만두·물만두·밥
-라멘 대기가 길거나 부모님이 만두를 선호할 때. 마늘 없는 교자 선택 가능.</t>
+고기 저녁 자리가 없거나 부모님이 만두를 선호할 때. 마늘 없는 교자 선택 가능.</t>
         </is>
       </c>
       <c r="E17" s="49" t="n">
@@ -2893,7 +2897,7 @@
       </c>
       <c r="H21" s="40" t="inlineStr">
         <is>
-          <t>이름이 같은 다른 지점으로 바꾸지 않음. 10/1 저녁 이용 가능 여부를 확인한 경우에만 하야시다와 교체.</t>
+          <t>이름이 같은 다른 지점으로 바꾸지 않음. 10/1 저녁 이용 가능 여부를 확인한 경우에만 고기 저녁 대신 고려.</t>
         </is>
       </c>
       <c r="I21" s="40" t="inlineStr">

</xml_diff>

<commit_message>
Tokyo guide: workbook row 7 map and source links point at Ushigoro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AoPkjGThxHgQ4GKNLnhfKD
</commit_message>
<xml_diff>
--- a/tokyo/tokyo-family-final.xlsx
+++ b/tokyo/tokyo-family-final.xlsx
@@ -2039,7 +2039,7 @@
       </c>
       <c r="J7" s="31" t="inlineStr">
         <is>
-          <t>원본 지도</t>
+          <t>지도 검색</t>
         </is>
       </c>
       <c r="K7" s="31" t="inlineStr">
@@ -2047,7 +2047,11 @@
           <t>출처 보기</t>
         </is>
       </c>
-      <c r="L7" s="31" t="n"/>
+      <c r="L7" s="35" t="inlineStr">
+        <is>
+          <t>대조 보기</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="142" customHeight="1">
       <c r="A8" s="15" t="n">
@@ -3401,69 +3405,70 @@
     <mergeCell ref="A4:L4"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" display="원본 지도" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" display="출처 보기" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" display="지도 검색" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" display="출처 보기" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" display="대조 보기" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" display="지도 검색" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" display="출처 보기" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" display="원본 지도" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" display="출처 보기" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" display="대조 보기" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" display="원본 지도" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" display="출처 보기" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" display="지도 검색" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" display="출처 보기" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" display="대조 보기" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" display="원본 지도" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" display="출처 보기" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" display="대조 보기" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" display="원본 지도" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" display="출처 보기" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" display="지도 검색" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" display="출처 보기" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" display="원본 지도" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" display="출처 보기" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" display="대조 보기" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" display="지도 검색" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" display="출처 보기" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" display="원본 지도" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" display="출처 보기" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" display="대조 보기" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" display="원본 지도" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" display="출처 보기" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" display="대조 보기" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" display="원본 지도" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" display="출처 보기" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" display="대조 보기" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" display="지도 검색" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" display="출처 보기" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" display="대조 보기" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" display="지도 검색" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" display="출처 보기" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" display="대조 보기" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" display="지도 검색" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" display="출처 보기" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" display="대조 보기" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" display="지도 검색" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" display="출처 보기" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" display="대조 보기" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" display="지도 검색" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" display="출처 보기" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" display="대조 보기" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" display="지도 검색" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" display="출처 보기" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" display="대조 보기" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" display="메뉴 PDF" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" display="행사 일정" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J8" display="지도 검색" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" display="출처 보기" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" display="대조 보기" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J10" display="지도 검색" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" display="출처 보기" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J11" display="원본 지도" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" display="출처 보기" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" display="대조 보기" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J12" display="원본 지도" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" display="출처 보기" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J13" display="지도 검색" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" display="출처 보기" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" display="대조 보기" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J14" display="원본 지도" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" display="출처 보기" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" display="대조 보기" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J15" display="원본 지도" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" display="출처 보기" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J16" display="지도 검색" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" display="출처 보기" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J17" display="원본 지도" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" display="출처 보기" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" display="대조 보기" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J18" display="지도 검색" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" display="출처 보기" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J19" display="원본 지도" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" display="출처 보기" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" display="대조 보기" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J20" display="원본 지도" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" display="출처 보기" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" display="대조 보기" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J21" display="원본 지도" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" display="출처 보기" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" display="대조 보기" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J22" display="지도 검색" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" display="출처 보기" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" display="대조 보기" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J23" display="지도 검색" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" display="출처 보기" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" display="대조 보기" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J24" display="지도 검색" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" display="출처 보기" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" display="대조 보기" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J25" display="지도 검색" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" display="출처 보기" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" display="대조 보기" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J26" display="지도 검색" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" display="출처 보기" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" display="대조 보기" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J27" display="지도 검색" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K27" display="출처 보기" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" display="대조 보기" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K31" display="메뉴 PDF" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" display="행사 일정" r:id="rId60"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId60"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId61"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>